<commit_message>
fix: make brb-dnra sheet consistent
</commit_message>
<xml_diff>
--- a/india_compliance/gst_india/data/gstr2b_excel_template_v1.1.xlsx
+++ b/india_compliance/gst_india/data/gstr2b_excel_template_v1.1.xlsx
@@ -907,7 +907,6 @@
       <c r="E9" s="43" t="n"/>
       <c r="F9" s="42" t="n"/>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
@@ -9560,8 +9559,8 @@
     <mergeCell ref="N5:N6"/>
     <mergeCell ref="A1:N3"/>
     <mergeCell ref="A4:N4"/>
+    <mergeCell ref="M5:M6"/>
     <mergeCell ref="C5:C6"/>
-    <mergeCell ref="M5:M6"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="B5:B6"/>
@@ -9800,8 +9799,8 @@
     <mergeCell ref="A1:Q3"/>
     <mergeCell ref="K6:N6"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:A7"/>
     <mergeCell ref="A4:Q4"/>
+    <mergeCell ref="F6:F7"/>
     <mergeCell ref="H6:H7"/>
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="I6:I7"/>
@@ -9814,7 +9813,7 @@
     <mergeCell ref="D6:D7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="D5:Q5"/>
-    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="A6:A7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
@@ -12142,14 +12141,14 @@
           <t>Taxable Value (₹)</t>
         </is>
       </c>
-      <c r="O6" s="43" t="n"/>
+      <c r="O6" s="26" t="inlineStr">
+        <is>
+          <t>Tax Amount</t>
+        </is>
+      </c>
       <c r="P6" s="43" t="n"/>
-      <c r="Q6" s="42" t="n"/>
-      <c r="R6" s="26" t="inlineStr">
-        <is>
-          <t>Tax Amount</t>
-        </is>
-      </c>
+      <c r="Q6" s="43" t="n"/>
+      <c r="R6" s="42" t="n"/>
       <c r="S6" s="26" t="inlineStr">
         <is>
           <t>GSTR-1/IFF Period</t>
@@ -12210,27 +12209,27 @@
       <c r="K7" s="45" t="n"/>
       <c r="L7" s="45" t="n"/>
       <c r="M7" s="45" t="n"/>
-      <c r="N7" s="26" t="inlineStr">
+      <c r="N7" s="45" t="n"/>
+      <c r="O7" s="26" t="inlineStr">
         <is>
           <t>Integrated Tax(₹)</t>
         </is>
       </c>
-      <c r="O7" s="26" t="inlineStr">
+      <c r="P7" s="26" t="inlineStr">
         <is>
           <t>Central Tax(₹)</t>
         </is>
       </c>
-      <c r="P7" s="26" t="inlineStr">
+      <c r="Q7" s="26" t="inlineStr">
         <is>
           <t>State/UT Tax(₹)</t>
         </is>
       </c>
-      <c r="Q7" s="26" t="inlineStr">
+      <c r="R7" s="26" t="inlineStr">
         <is>
           <t>Cess(₹)</t>
         </is>
       </c>
-      <c r="R7" s="45" t="n"/>
       <c r="S7" s="45" t="n"/>
       <c r="T7" s="45" t="n"/>
       <c r="U7" s="45" t="n"/>
@@ -12239,9 +12238,7 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="N6:Q6"/>
     <mergeCell ref="F6:J6"/>
-    <mergeCell ref="R6:R7"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A4:V4"/>
     <mergeCell ref="V6:V7"/>
@@ -12249,11 +12246,13 @@
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="M6:M7"/>
     <mergeCell ref="E6:E7"/>
+    <mergeCell ref="O6:R6"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="S6:S7"/>
     <mergeCell ref="D6:D7"/>
     <mergeCell ref="A1:V3"/>
     <mergeCell ref="L6:L7"/>
+    <mergeCell ref="N6:N7"/>
     <mergeCell ref="T6:T7"/>
     <mergeCell ref="K6:K7"/>
     <mergeCell ref="C6:C7"/>
@@ -12753,9 +12752,9 @@
   <mergeCells count="16">
     <mergeCell ref="C5:R5"/>
     <mergeCell ref="K6:N6"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="I6:I7"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="E6:H6"/>
     <mergeCell ref="J6:J7"/>
     <mergeCell ref="P6:P7"/>
     <mergeCell ref="R6:R7"/>
@@ -13953,8 +13952,8 @@
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="A1:M3"/>
     <mergeCell ref="A4:M4"/>
+    <mergeCell ref="M5:M6"/>
     <mergeCell ref="C5:C6"/>
-    <mergeCell ref="M5:M6"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="B5:B6"/>

</xml_diff>